<commit_message>
Created decoder5 - matching IDL data
</commit_message>
<xml_diff>
--- a/Decoder Ring.xlsx
+++ b/Decoder Ring.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d9622e146f2de41c/Documents/GitHub/DataFlow/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cohrinc-my.sharepoint.com/personal/dennis_rossman_coherent_com/Documents/Documents/GitHub/DataFlow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="320" documentId="8_{7C37ACB5-38B9-42B1-AAF6-47486B393A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07CB879C-D734-4282-904C-2DBF1F1A7A87}"/>
+  <xr:revisionPtr revIDLastSave="323" documentId="8_{7C37ACB5-38B9-42B1-AAF6-47486B393A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF3B20D3-BCB0-47D5-A32A-D0139F3E87CA}"/>
   <bookViews>
-    <workbookView xWindow="30615" yWindow="675" windowWidth="26985" windowHeight="22500" activeTab="2" xr2:uid="{D3089677-3F36-4795-9B26-0BDE8E67A95B}"/>
+    <workbookView minimized="1" xWindow="15" yWindow="15" windowWidth="28770" windowHeight="15420" activeTab="2" xr2:uid="{D3089677-3F36-4795-9B26-0BDE8E67A95B}"/>
   </bookViews>
   <sheets>
     <sheet name="Logic Analyzer" sheetId="7" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="436">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -1141,9 +1141,6 @@
     <t>Implant state</t>
   </si>
   <si>
-    <t>5 = waiting/standby, 11 = pump down (pump down ends when the state changes from 11), implant starts at 3 (getting ready?), then state 1, then 2, then 3,  State 6 is hold?</t>
-  </si>
-  <si>
     <t>Data is weird.  There is data between 5 and 25 with most around 10, then nothing until 246 up to 250?</t>
   </si>
   <si>
@@ -1337,6 +1334,15 @@
   </si>
   <si>
     <t>The number drops to 3 and the actual time drops to 0 - pump down ended, waiting for implant start</t>
+  </si>
+  <si>
+    <t>Good finding, if you take the time from an IDL file, that is the completion time of the implant.  You can then add the milliseconds</t>
+  </si>
+  <si>
+    <t>from the Arduino and predict all of the other IDL finish times from the same file.</t>
+  </si>
+  <si>
+    <t>5 = waiting/standby, 11 = pump down (pump down ends when the state changes from 11 usually goes to 3 or 4, not sure the significance), 3 or 4 is waiting for implant to start?, then state 1, then 2, then 3 are the beginning, middle, end data - these seem to correlate to DataFlow,  State 6 is hold?</t>
   </si>
 </sst>
 </file>
@@ -2066,6 +2072,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2384,44 +2394,44 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BA9EF41-673D-434C-8874-313FFF75849C}">
   <dimension ref="A1:Z58"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="U5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="21:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="21:21" x14ac:dyDescent="0.3">
       <c r="U24" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="40" spans="26:26" x14ac:dyDescent="0.25">
+    <row r="40" spans="26:26" x14ac:dyDescent="0.3">
       <c r="Z40" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>33</v>
       </c>
@@ -2435,35 +2445,35 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D21FFDC-D4C9-49CE-97EF-F91F73D1EB22}">
   <dimension ref="A1:N331"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
     <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>199</v>
       </c>
@@ -2489,7 +2499,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>22</v>
       </c>
@@ -2518,7 +2528,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>22</v>
       </c>
@@ -2547,7 +2557,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>22</v>
       </c>
@@ -2576,7 +2586,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>22</v>
       </c>
@@ -2605,22 +2615,22 @@
         <v>298</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>199</v>
       </c>
@@ -2640,7 +2650,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>22</v>
       </c>
@@ -2666,7 +2676,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>22</v>
       </c>
@@ -2692,7 +2702,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>22</v>
       </c>
@@ -2718,7 +2728,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>22</v>
       </c>
@@ -2744,52 +2754,52 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>199</v>
       </c>
@@ -2833,7 +2843,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>22</v>
       </c>
@@ -2859,12 +2869,12 @@
         <v>255</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>22</v>
       </c>
@@ -2896,7 +2906,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>22</v>
       </c>
@@ -2925,7 +2935,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>22</v>
       </c>
@@ -2954,247 +2964,247 @@
         <v>301</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="86" spans="1:1" ht="21" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A86" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>201</v>
       </c>
@@ -3205,7 +3215,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>49</v>
       </c>
@@ -3216,7 +3226,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>50</v>
       </c>
@@ -3227,17 +3237,17 @@
         <v>205</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>74</v>
       </c>
@@ -3248,7 +3258,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>75</v>
       </c>
@@ -3259,37 +3269,37 @@
         <v>206</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>74</v>
       </c>
@@ -3297,7 +3307,7 @@
         <v>1.3332999999999999</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>75</v>
       </c>
@@ -3305,42 +3315,42 @@
         <v>64</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>74</v>
       </c>
@@ -3348,7 +3358,7 @@
         <v>3.125038028597505E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>75</v>
       </c>
@@ -3356,17 +3366,17 @@
         <v>61</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>0</v>
       </c>
@@ -3377,7 +3387,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>1</v>
       </c>
@@ -3388,7 +3398,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>2</v>
       </c>
@@ -3399,7 +3409,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>3</v>
       </c>
@@ -3413,7 +3423,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>4</v>
       </c>
@@ -3427,7 +3437,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>5</v>
       </c>
@@ -3438,7 +3448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>6</v>
       </c>
@@ -3449,7 +3459,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>7</v>
       </c>
@@ -3457,7 +3467,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>8</v>
       </c>
@@ -3468,7 +3478,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>9</v>
       </c>
@@ -3479,7 +3489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>10</v>
       </c>
@@ -3490,7 +3500,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>11</v>
       </c>
@@ -3498,7 +3508,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>12</v>
       </c>
@@ -3512,7 +3522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>13</v>
       </c>
@@ -3526,7 +3536,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>14</v>
       </c>
@@ -3537,7 +3547,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>15</v>
       </c>
@@ -3548,7 +3558,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>16</v>
       </c>
@@ -3559,7 +3569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>17</v>
       </c>
@@ -3570,7 +3580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>18</v>
       </c>
@@ -3584,7 +3594,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>19</v>
       </c>
@@ -3595,7 +3605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>20</v>
       </c>
@@ -3606,7 +3616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>21</v>
       </c>
@@ -3614,7 +3624,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>22</v>
       </c>
@@ -3628,17 +3638,17 @@
         <v>79</v>
       </c>
     </row>
-    <row r="165" spans="1:4" ht="21" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A165" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>0</v>
       </c>
@@ -3649,7 +3659,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>1</v>
       </c>
@@ -3660,7 +3670,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>2</v>
       </c>
@@ -3671,7 +3681,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>3</v>
       </c>
@@ -3685,7 +3695,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>4</v>
       </c>
@@ -3699,7 +3709,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>5</v>
       </c>
@@ -3710,7 +3720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>6</v>
       </c>
@@ -3721,7 +3731,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>10</v>
       </c>
@@ -3732,7 +3742,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>14</v>
       </c>
@@ -3743,7 +3753,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>18</v>
       </c>
@@ -3754,7 +3764,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>22</v>
       </c>
@@ -3765,7 +3775,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>26</v>
       </c>
@@ -3776,7 +3786,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>30</v>
       </c>
@@ -3787,7 +3797,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>193</v>
       </c>
@@ -3798,7 +3808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>38</v>
       </c>
@@ -3809,7 +3819,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>42</v>
       </c>
@@ -3820,7 +3830,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>46</v>
       </c>
@@ -3831,7 +3841,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>50</v>
       </c>
@@ -3842,7 +3852,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>54</v>
       </c>
@@ -3853,7 +3863,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>58</v>
       </c>
@@ -3864,7 +3874,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>62</v>
       </c>
@@ -3875,7 +3885,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>66</v>
       </c>
@@ -3886,7 +3896,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>70</v>
       </c>
@@ -3897,7 +3907,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>74</v>
       </c>
@@ -3908,7 +3918,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>78</v>
       </c>
@@ -3919,7 +3929,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>82</v>
       </c>
@@ -3930,7 +3940,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>86</v>
       </c>
@@ -3941,7 +3951,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>90</v>
       </c>
@@ -3952,7 +3962,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>94</v>
       </c>
@@ -3963,7 +3973,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>194</v>
       </c>
@@ -3974,7 +3984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>114</v>
       </c>
@@ -3985,7 +3995,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>118</v>
       </c>
@@ -3996,7 +4006,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>195</v>
       </c>
@@ -4007,7 +4017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>126</v>
       </c>
@@ -4018,7 +4028,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>130</v>
       </c>
@@ -4029,7 +4039,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>196</v>
       </c>
@@ -4040,7 +4050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>150</v>
       </c>
@@ -4051,7 +4061,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>154</v>
       </c>
@@ -4062,7 +4072,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>197</v>
       </c>
@@ -4073,7 +4083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>166</v>
       </c>
@@ -4084,7 +4094,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>170</v>
       </c>
@@ -4095,7 +4105,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>174</v>
       </c>
@@ -4106,7 +4116,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>178</v>
       </c>
@@ -4117,7 +4127,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>182</v>
       </c>
@@ -4128,7 +4138,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>186</v>
       </c>
@@ -4139,7 +4149,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>190</v>
       </c>
@@ -4150,7 +4160,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>194</v>
       </c>
@@ -4161,7 +4171,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>198</v>
       </c>
@@ -4172,7 +4182,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>202</v>
       </c>
@@ -4183,7 +4193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>203</v>
       </c>
@@ -4191,7 +4201,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>204</v>
       </c>
@@ -4202,17 +4212,17 @@
         <v>255</v>
       </c>
     </row>
-    <row r="221" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:3" ht="21" x14ac:dyDescent="0.4">
       <c r="A221" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>0</v>
       </c>
@@ -4223,7 +4233,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>1</v>
       </c>
@@ -4234,7 +4244,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>2</v>
       </c>
@@ -4245,7 +4255,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>3</v>
       </c>
@@ -4259,7 +4269,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>4</v>
       </c>
@@ -4273,7 +4283,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>5</v>
       </c>
@@ -4284,7 +4294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>6</v>
       </c>
@@ -4295,7 +4305,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>10</v>
       </c>
@@ -4306,7 +4316,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>14</v>
       </c>
@@ -4317,7 +4327,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>18</v>
       </c>
@@ -4328,7 +4338,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>22</v>
       </c>
@@ -4339,7 +4349,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>26</v>
       </c>
@@ -4350,7 +4360,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>30</v>
       </c>
@@ -4361,7 +4371,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>34</v>
       </c>
@@ -4372,7 +4382,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>38</v>
       </c>
@@ -4383,7 +4393,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>42</v>
       </c>
@@ -4391,7 +4401,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>43</v>
       </c>
@@ -4402,17 +4412,17 @@
         <v>255</v>
       </c>
     </row>
-    <row r="243" spans="1:4" ht="21" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A243" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>0</v>
       </c>
@@ -4423,7 +4433,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>1</v>
       </c>
@@ -4434,7 +4444,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>2</v>
       </c>
@@ -4445,7 +4455,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>3</v>
       </c>
@@ -4459,7 +4469,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>4</v>
       </c>
@@ -4473,7 +4483,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>5</v>
       </c>
@@ -4484,7 +4494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>6</v>
       </c>
@@ -4495,7 +4505,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>10</v>
       </c>
@@ -4506,7 +4516,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>14</v>
       </c>
@@ -4517,7 +4527,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>18</v>
       </c>
@@ -4528,7 +4538,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>22</v>
       </c>
@@ -4539,7 +4549,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>227</v>
       </c>
@@ -4550,7 +4560,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>32</v>
       </c>
@@ -4558,7 +4568,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="259" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>33</v>
       </c>
@@ -4569,17 +4579,17 @@
         <v>255</v>
       </c>
     </row>
-    <row r="262" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="264" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A264" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="266" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A266" s="6" t="s">
         <v>271</v>
       </c>
@@ -4587,7 +4597,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="267" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>269</v>
       </c>
@@ -4613,7 +4623,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="268" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>90678</v>
       </c>
@@ -4641,7 +4651,7 @@
         <v>8.8224266084386513E-5</v>
       </c>
     </row>
-    <row r="269" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C269">
         <v>74</v>
       </c>
@@ -4665,18 +4675,18 @@
         <v>0.99991167833248695</v>
       </c>
     </row>
-    <row r="270" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D270" s="4"/>
       <c r="F270" s="4"/>
       <c r="H270" s="4"/>
       <c r="L270" s="4"/>
     </row>
-    <row r="271" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A271" s="7" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="273" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A273" s="6" t="s">
         <v>275</v>
       </c>
@@ -4684,7 +4694,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="274" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>269</v>
       </c>
@@ -4710,7 +4720,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="275" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>22476</v>
       </c>
@@ -4738,7 +4748,7 @@
         <v>2.0688734650293646E-2</v>
       </c>
     </row>
-    <row r="276" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C276">
         <v>16</v>
       </c>
@@ -4762,12 +4772,12 @@
         <v>0.95996556177356862</v>
       </c>
     </row>
-    <row r="278" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A278" s="7" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="280" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A280" s="6" t="s">
         <v>276</v>
       </c>
@@ -4775,7 +4785,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="281" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>269</v>
       </c>
@@ -4801,7 +4811,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="282" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>90705</v>
       </c>
@@ -4829,7 +4839,7 @@
         <v>6.9455928559616334E-4</v>
       </c>
     </row>
-    <row r="283" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C283">
         <v>9</v>
       </c>
@@ -4853,7 +4863,7 @@
         <v>0.9993054330569765</v>
       </c>
     </row>
-    <row r="284" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C284">
         <v>21</v>
       </c>
@@ -4865,25 +4875,25 @@
         <v>8.8198004520147736E-5</v>
       </c>
     </row>
-    <row r="286" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="288" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A288" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="289" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A289" s="7"/>
     </row>
-    <row r="290" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A290" s="6" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="291" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>269</v>
       </c>
@@ -4897,7 +4907,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="292" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>90678</v>
       </c>
@@ -4915,7 +4925,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="293" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C293">
         <v>74</v>
       </c>
@@ -4931,20 +4941,20 @@
         <v>278</v>
       </c>
     </row>
-    <row r="294" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D294" s="4"/>
       <c r="F294" s="4"/>
       <c r="H294" s="4"/>
       <c r="L294" s="4"/>
     </row>
-    <row r="295" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A295" s="6" t="s">
         <v>272</v>
       </c>
       <c r="H295" s="4"/>
       <c r="L295" s="4"/>
     </row>
-    <row r="296" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>269</v>
       </c>
@@ -4960,7 +4970,7 @@
       <c r="H296" s="4"/>
       <c r="L296" s="4"/>
     </row>
-    <row r="297" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>90578</v>
       </c>
@@ -4980,7 +4990,7 @@
       <c r="H297" s="4"/>
       <c r="L297" s="4"/>
     </row>
-    <row r="298" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B298" s="4"/>
       <c r="C298">
         <v>205</v>
@@ -4995,17 +5005,17 @@
       <c r="H298" s="4"/>
       <c r="L298" s="4"/>
     </row>
-    <row r="299" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A299" s="7" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="301" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A301" s="6" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="302" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>269</v>
       </c>
@@ -5019,7 +5029,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="303" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>22476</v>
       </c>
@@ -5037,7 +5047,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="304" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C304">
         <v>16</v>
       </c>
@@ -5053,12 +5063,12 @@
         <v>280</v>
       </c>
     </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A306" s="6" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>269</v>
       </c>
@@ -5072,7 +5082,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>11615</v>
       </c>
@@ -5090,7 +5100,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B309" s="4"/>
       <c r="C309">
         <v>34</v>
@@ -5103,17 +5113,17 @@
         <v>0.95996556177356862</v>
       </c>
     </row>
-    <row r="311" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A311" s="7" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="313" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A313" s="6" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="314" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>269</v>
       </c>
@@ -5127,7 +5137,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="315" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>90705</v>
       </c>
@@ -5145,7 +5155,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="316" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C316">
         <v>9</v>
       </c>
@@ -5161,7 +5171,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="317" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C317">
         <v>21</v>
       </c>
@@ -5173,12 +5183,12 @@
         <v>8.8198004520147736E-5</v>
       </c>
     </row>
-    <row r="319" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A319" s="6" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="320" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>269</v>
       </c>
@@ -5192,7 +5202,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="321" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>90704</v>
       </c>
@@ -5210,7 +5220,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="322" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B322" s="4"/>
       <c r="C322">
         <v>44</v>
@@ -5223,22 +5233,22 @@
         <v>0.9993054330569765</v>
       </c>
     </row>
-    <row r="326" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A326" s="7" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="327" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="328" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="330" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>14</v>
       </c>
@@ -5273,7 +5283,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="331" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>288</v>
       </c>
@@ -5317,21 +5327,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FA6E082-610D-4F78-9F07-30C3D4CB5C68}">
-  <dimension ref="A1:E101"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E104"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
-    <col min="4" max="4" width="30.28515625" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.5546875" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="30.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>83</v>
       </c>
@@ -5345,7 +5355,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>84</v>
       </c>
@@ -5356,7 +5366,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>85</v>
       </c>
@@ -5367,7 +5377,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>86</v>
       </c>
@@ -5378,7 +5388,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>87</v>
       </c>
@@ -5389,7 +5399,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>88</v>
       </c>
@@ -5400,7 +5410,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>89</v>
       </c>
@@ -5411,7 +5421,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>90</v>
       </c>
@@ -5422,9 +5432,9 @@
         <v>238</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B11" t="s">
         <v>83</v>
@@ -5433,10 +5443,10 @@
         <v>364</v>
       </c>
       <c r="D11" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>367</v>
       </c>
@@ -5447,10 +5457,10 @@
         <v>365</v>
       </c>
       <c r="D12" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>351</v>
       </c>
@@ -5464,7 +5474,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -5481,7 +5491,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -5492,7 +5502,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>91</v>
       </c>
@@ -5506,9 +5516,9 @@
         <v>350</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B18" t="s">
         <v>18</v>
@@ -5520,9 +5530,9 @@
         <v>353</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B19" t="s">
         <v>18</v>
@@ -5534,7 +5544,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>92</v>
       </c>
@@ -5548,7 +5558,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>93</v>
       </c>
@@ -5559,7 +5569,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>94</v>
       </c>
@@ -5570,7 +5580,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>95</v>
       </c>
@@ -5581,7 +5591,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>96</v>
       </c>
@@ -5592,9 +5602,9 @@
         <v>235</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B26" t="s">
         <v>229</v>
@@ -5603,12 +5613,12 @@
         <v>236</v>
       </c>
       <c r="D26" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B27" t="s">
         <v>229</v>
@@ -5620,9 +5630,9 @@
         <v>362</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B28" t="s">
         <v>229</v>
@@ -5634,8 +5644,8 @@
         <v>363</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" ht="13.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>97</v>
       </c>
@@ -5649,7 +5659,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>99</v>
       </c>
@@ -5660,7 +5670,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>119</v>
       </c>
@@ -5671,7 +5681,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>120</v>
       </c>
@@ -5682,7 +5692,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>121</v>
       </c>
@@ -5693,7 +5703,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>122</v>
       </c>
@@ -5704,9 +5714,9 @@
         <v>236</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B36" t="s">
         <v>239</v>
@@ -5715,12 +5725,12 @@
         <v>237</v>
       </c>
       <c r="D36" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B37" t="s">
         <v>239</v>
@@ -5729,10 +5739,10 @@
         <v>238</v>
       </c>
       <c r="D37" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>98</v>
       </c>
@@ -5743,7 +5753,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>100</v>
       </c>
@@ -5754,35 +5764,35 @@
         <v>254</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B40" t="s">
         <v>239</v>
       </c>
       <c r="C40" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="D40" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B41" t="s">
         <v>239</v>
       </c>
       <c r="C41" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D41" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>123</v>
       </c>
@@ -5793,7 +5803,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>126</v>
       </c>
@@ -5804,7 +5814,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>103</v>
       </c>
@@ -5815,7 +5825,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>104</v>
       </c>
@@ -5826,7 +5836,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>101</v>
       </c>
@@ -5837,7 +5847,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>106</v>
       </c>
@@ -5848,7 +5858,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>108</v>
       </c>
@@ -5859,7 +5869,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>109</v>
       </c>
@@ -5870,7 +5880,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>110</v>
       </c>
@@ -5881,91 +5891,91 @@
         <v>263</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B51" t="s">
         <v>239</v>
       </c>
       <c r="C51" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D51" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B52" t="s">
         <v>239</v>
       </c>
       <c r="C52" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="D52" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B53" t="s">
         <v>239</v>
       </c>
       <c r="C53" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D53" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B54" t="s">
         <v>239</v>
       </c>
       <c r="C54" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D54" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B55" t="s">
         <v>239</v>
       </c>
       <c r="C55" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D55" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B56" t="s">
         <v>239</v>
       </c>
       <c r="C56" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D56" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>105</v>
       </c>
@@ -5976,7 +5986,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>124</v>
       </c>
@@ -5987,21 +5997,21 @@
         <v>246</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B59" t="s">
         <v>239</v>
       </c>
       <c r="C59" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D59" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>111</v>
       </c>
@@ -6012,7 +6022,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>112</v>
       </c>
@@ -6023,21 +6033,21 @@
         <v>248</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B62" t="s">
         <v>239</v>
       </c>
       <c r="C62" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D62" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>107</v>
       </c>
@@ -6048,38 +6058,38 @@
         <v>249</v>
       </c>
       <c r="D63" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B64" t="s">
         <v>239</v>
       </c>
       <c r="C64" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="D64" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B65" t="s">
         <v>239</v>
       </c>
       <c r="C65" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D65" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>114</v>
       </c>
@@ -6090,49 +6100,49 @@
         <v>250</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B67" t="s">
         <v>239</v>
       </c>
       <c r="C67" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="D67" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B68" t="s">
         <v>239</v>
       </c>
       <c r="C68" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D68" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B69" t="s">
         <v>239</v>
       </c>
       <c r="C69" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D69" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>118</v>
       </c>
@@ -6143,21 +6153,21 @@
         <v>251</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B71" t="s">
         <v>239</v>
       </c>
       <c r="C71" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D71" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>117</v>
       </c>
@@ -6168,7 +6178,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>113</v>
       </c>
@@ -6179,7 +6189,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>125</v>
       </c>
@@ -6190,21 +6200,21 @@
         <v>242</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B75" t="s">
         <v>239</v>
       </c>
       <c r="C75" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D75" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>115</v>
       </c>
@@ -6215,7 +6225,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>116</v>
       </c>
@@ -6226,7 +6236,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>102</v>
       </c>
@@ -6237,94 +6247,104 @@
         <v>241</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B89" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C90" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C91" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C94" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C95" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C95" t="s">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C96" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C96" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="97" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C97" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="98" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C98" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="99" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C99" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="100" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C100" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="101" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C101" t="s">
         <v>313</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>434</v>
       </c>
     </row>
   </sheetData>

</xml_diff>